<commit_message>
Derivados regenerados tras la actualizacion de eu-agrifood
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WpevEvgxxTSUSU4BwGMDZh
</commit_message>
<xml_diff>
--- a/data/pack/eu/azucar.xlsx
+++ b/data/pack/eu/azucar.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K241"/>
+  <dimension ref="A1:K243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13689,6 +13689,116 @@
         </is>
       </c>
       <c r="K241" t="inlineStr">
+        <is>
+          <t>Source: European Commission (Agri-food data portal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>azucar</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Azúcar</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="E242" t="n">
+        <v>499.4133</v>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>tonelada</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>European Commission — Agri-food Data Portal (DG AGRI)</t>
+        </is>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>EU-REUSE-2011-833</t>
+        </is>
+      </c>
+      <c r="K242" t="inlineStr">
+        <is>
+          <t>Source: European Commission (Agri-food data portal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>azucar</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Azúcar</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="E243" t="n">
+        <v>500.0078</v>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>tonelada</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>European Commission — Agri-food Data Portal (DG AGRI)</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>EU-REUSE-2011-833</t>
+        </is>
+      </c>
+      <c r="K243" t="inlineStr">
         <is>
           <t>Source: European Commission (Agri-food data portal)</t>
         </is>
@@ -13792,7 +13902,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>2026-06</t>
+          <t>2026-08</t>
         </is>
       </c>
     </row>
@@ -13803,7 +13913,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="9">
@@ -13898,7 +14008,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>

</xml_diff>